<commit_message>
Teach decoder the Alliance/IPSO (European) trailing-letter date code
Field test on three Czech-built Alliance washer-extractors exposed a gap:
IPSO/European units encode the date as a trailing [YearLetter][MonthLetter]
pair (e.g. …FH = Apr 2016, …MK = May 2019), not the US-domestic leading
YYMM. The decoder previously (correctly) abstained rather than misread the
leading "40…" as a year — now it decodes the trailing code at medium
confidence and flags it for Alliance validation.

- serialDecoder.js: alliance() tries the IPSO trailing-letter table first,
  then US-domestic YYMM, then legacy.
- brands.js: documents the IPSO format with real worked examples.
- Regenerated docs/ reference + vendor checklist.

US-domestic pilot unchanged at 100% precision (9/9); no regression.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Kn8R8jTNya2ZZLsLje6xJ
</commit_message>
<xml_diff>
--- a/docs/Serial-Decoding-Reference.xlsx
+++ b/docs/Serial-Decoding-Reference.xlsx
@@ -463,7 +463,7 @@
         <v>alliance</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -1905,7 +1905,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J27"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1959,7 +1959,7 @@
         <v>Commercial laundry</v>
       </c>
       <c r="C2" t="str">
-        <v>~mid-2000s–present</v>
+        <v>US-built (~mid-2000s–present)</v>
       </c>
       <c r="D2" t="str">
         <v>YYMMnnnnnn</v>
@@ -1977,7 +1977,7 @@
         <v>Yes</v>
       </c>
       <c r="I2" t="str">
-        <v>serial starts with a letter (legacy), or is &lt;4 digits</v>
+        <v>serial is neither US-domestic YYMM nor an IPSO trailing-letter code (verify with Alliance)</v>
       </c>
       <c r="J2" t="str">
         <v>https://homespy.io/alliance-laundry-serial-lookup | http://www.appliance411.com/service/date-code.php</v>
@@ -1991,16 +1991,16 @@
         <v>Commercial laundry</v>
       </c>
       <c r="C3" t="str">
-        <v>legacy (letter-suffix)</v>
+        <v>IPSO / European (Czech-built)</v>
       </c>
       <c r="D3" t="str">
-        <v>…+2 trailing letters</v>
+        <v>…[YearLetter][MonthLetter]</v>
       </c>
       <c r="E3" t="str">
-        <v>date is the LAST two letters (year letter cycles, month letter) — leading-digit rule does NOT apply</v>
+        <v>date is the LAST two letters: penultimate = year (cycles ~20 yrs: …D=2015,F=2016,H=2017,K=2018,M=2019,Q=2020), last = month (two letters/month: Apr=G/H, May=J/K, Nov=V/Y). Leading digits are a plant/sequence code, NOT the date</v>
       </c>
       <c r="F3" t="str">
-        <v>…DK → 2015-05</v>
+        <v>40F002829FH → Apr 2016; 40F003349MK → May 2019</v>
       </c>
       <c r="G3" t="str">
         <v>medium</v>
@@ -2017,34 +2017,34 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>AAON</v>
+        <v>Alliance / Unimac</v>
       </c>
       <c r="B4" t="str">
-        <v>HVAC (rooftop/DOAS)</v>
+        <v>Commercial laundry</v>
       </c>
       <c r="C4" t="str">
-        <v>Style 1</v>
+        <v>legacy US letter-prefixed</v>
       </c>
       <c r="D4" t="str">
-        <v>YYYYMM…</v>
+        <v>[letter]…</v>
       </c>
       <c r="E4" t="str">
-        <v>digits 1-4 = full year, 5-6 = month</v>
+        <v>leading-digit rule does not apply — verify</v>
       </c>
       <c r="F4" t="str">
-        <v>200108AKG… → Aug 2001</v>
+        <v>—</v>
       </c>
       <c r="G4" t="str">
-        <v>high</v>
+        <v>low</v>
       </c>
       <c r="H4" t="str">
         <v>Yes</v>
       </c>
       <c r="I4" t="str">
-        <v>serial shape matches none of AAON’s 3 styles</v>
+        <v/>
       </c>
       <c r="J4" t="str">
-        <v>https://www.building-center.org/aaon-hvac-age/ | https://www.stewartchi.com/aaon.html</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -2055,60 +2055,60 @@
         <v>HVAC (rooftop/DOAS)</v>
       </c>
       <c r="C5" t="str">
-        <v>Style 2</v>
+        <v>Style 1</v>
       </c>
       <c r="D5" t="str">
-        <v>YY…</v>
+        <v>YYYYMM…</v>
       </c>
       <c r="E5" t="str">
-        <v>digits 1-2 = year (2-digit)</v>
+        <v>digits 1-4 = full year, 5-6 = month</v>
       </c>
       <c r="F5" t="str">
-        <v>160901518 → 2016</v>
+        <v>200108AKG… → Aug 2001</v>
       </c>
       <c r="G5" t="str">
-        <v>medium</v>
+        <v>high</v>
       </c>
       <c r="H5" t="str">
         <v>Yes</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>serial shape matches none of AAON’s 3 styles</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>https://www.building-center.org/aaon-hvac-age/ | https://www.stewartchi.com/aaon.html</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>A. O. Smith</v>
+        <v>AAON</v>
       </c>
       <c r="B6" t="str">
-        <v>Water heaters</v>
+        <v>HVAC (rooftop/DOAS)</v>
       </c>
       <c r="C6" t="str">
-        <v>~2008–present</v>
+        <v>Style 2</v>
       </c>
       <c r="D6" t="str">
-        <v>YYWWnnnnnn</v>
+        <v>YY…</v>
       </c>
       <c r="E6" t="str">
-        <v>digits 1-2 = year, 3-4 = week (01-52)</v>
+        <v>digits 1-2 = year (2-digit)</v>
       </c>
       <c r="F6" t="str">
-        <v>2108… → wk8 2021</v>
+        <v>160901518 → 2016</v>
       </c>
       <c r="G6" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="H6" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="I6" t="str">
-        <v>prefix is not YYWW / MMYY / letter+YY</v>
+        <v/>
       </c>
       <c r="J6" t="str">
-        <v>https://inspectapedia.com/plumbing/AO-Smith-Water-Heater-Age-Manuals.php | https://www.building-center.org/a-o-smith-water-heater-age/</v>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -2119,48 +2119,48 @@
         <v>Water heaters</v>
       </c>
       <c r="C7" t="str">
-        <v>pre-2008 letter</v>
+        <v>~2008–present</v>
       </c>
       <c r="D7" t="str">
-        <v>[MonthLetter]YY…</v>
+        <v>YYWWnnnnnn</v>
       </c>
       <c r="E7" t="str">
-        <v>letter = month (A=Jan…M=Dec, no I), next 2 digits = year</v>
+        <v>digits 1-2 = year, 3-4 = week (01-52)</v>
       </c>
       <c r="F7" t="str">
-        <v>B01… → Feb 2001</v>
+        <v>2108… → wk8 2021</v>
       </c>
       <c r="G7" t="str">
-        <v>medium</v>
+        <v>high</v>
       </c>
       <c r="H7" t="str">
         <v>No</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>prefix is not YYWW / MMYY / letter+YY</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>https://inspectapedia.com/plumbing/AO-Smith-Water-Heater-Age-Manuals.php | https://www.building-center.org/a-o-smith-water-heater-age/</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>State Water Heaters</v>
+        <v>A. O. Smith</v>
       </c>
       <c r="B8" t="str">
         <v>Water heaters</v>
       </c>
       <c r="C8" t="str">
-        <v>~2008–present</v>
+        <v>pre-2008 letter</v>
       </c>
       <c r="D8" t="str">
-        <v>YYWW…</v>
+        <v>[MonthLetter]YY…</v>
       </c>
       <c r="E8" t="str">
-        <v>A.O. Smith family scheme: digits 1-2 = year, 3-4 = week</v>
+        <v>letter = month (A=Jan…M=Dec, no I), next 2 digits = year</v>
       </c>
       <c r="F8" t="str">
-        <v>1523… → wk23 2015</v>
+        <v>B01… → Feb 2001</v>
       </c>
       <c r="G8" t="str">
         <v>medium</v>
@@ -2169,10 +2169,10 @@
         <v>No</v>
       </c>
       <c r="I8" t="str">
-        <v>prefix not YYWW / letter+YY</v>
+        <v/>
       </c>
       <c r="J8" t="str">
-        <v>https://www.building-center.org/state-water-heater-age/</v>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -2183,16 +2183,16 @@
         <v>Water heaters</v>
       </c>
       <c r="C9" t="str">
-        <v>legacy</v>
+        <v>~2008–present</v>
       </c>
       <c r="D9" t="str">
-        <v>[MonthLetter]YY…</v>
+        <v>YYWW…</v>
       </c>
       <c r="E9" t="str">
-        <v>letter = month, next 2 digits = year</v>
+        <v>A.O. Smith family scheme: digits 1-2 = year, 3-4 = week</v>
       </c>
       <c r="F9" t="str">
-        <v>C05… → Mar 2005</v>
+        <v>1523… → wk23 2015</v>
       </c>
       <c r="G9" t="str">
         <v>medium</v>
@@ -2201,30 +2201,30 @@
         <v>No</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>prefix not YYWW / letter+YY</v>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>https://www.building-center.org/state-water-heater-age/</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Raypak</v>
+        <v>State Water Heaters</v>
       </c>
       <c r="B10" t="str">
-        <v>Boilers / pool heaters</v>
+        <v>Water heaters</v>
       </c>
       <c r="C10" t="str">
-        <v>1995–present</v>
+        <v>legacy</v>
       </c>
       <c r="D10" t="str">
-        <v>YYMMnnnnnn (10-digit)</v>
+        <v>[MonthLetter]YY…</v>
       </c>
       <c r="E10" t="str">
-        <v>digits 1-2 = year, 3-4 = month</v>
+        <v>letter = month, next 2 digits = year</v>
       </c>
       <c r="F10" t="str">
-        <v>1604304448 → Apr 2016</v>
+        <v>C05… → Mar 2005</v>
       </c>
       <c r="G10" t="str">
         <v>medium</v>
@@ -2233,10 +2233,10 @@
         <v>No</v>
       </c>
       <c r="I10" t="str">
-        <v>first 4 digits give no valid month in either order</v>
+        <v/>
       </c>
       <c r="J10" t="str">
-        <v>https://www.building-center.org/raypak-hvac-age/ | https://www.raypak.com/how-to-read-a-raypak-model-number/</v>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -2247,60 +2247,60 @@
         <v>Boilers / pool heaters</v>
       </c>
       <c r="C11" t="str">
-        <v>pre-1995</v>
+        <v>1995–present</v>
       </c>
       <c r="D11" t="str">
-        <v>MMYY…</v>
+        <v>YYMMnnnnnn (10-digit)</v>
       </c>
       <c r="E11" t="str">
-        <v>field order reversed (month then year)</v>
+        <v>digits 1-2 = year, 3-4 = month</v>
       </c>
       <c r="F11" t="str">
-        <v>0192… → Jan 1992</v>
+        <v>1604304448 → Apr 2016</v>
       </c>
       <c r="G11" t="str">
-        <v>low</v>
+        <v>medium</v>
       </c>
       <c r="H11" t="str">
         <v>No</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>first 4 digits give no valid month in either order</v>
       </c>
       <c r="J11" t="str">
-        <v/>
+        <v>https://www.building-center.org/raypak-hvac-age/ | https://www.raypak.com/how-to-read-a-raypak-model-number/</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Trane</v>
+        <v>Raypak</v>
       </c>
       <c r="B12" t="str">
-        <v>HVAC</v>
+        <v>Boilers / pool heaters</v>
       </c>
       <c r="C12" t="str">
-        <v>2010–present</v>
+        <v>pre-1995</v>
       </c>
       <c r="D12" t="str">
-        <v>YYWW…</v>
+        <v>MMYY…</v>
       </c>
       <c r="E12" t="str">
-        <v>digits 1-2 = year, 3-4 = week</v>
+        <v>field order reversed (month then year)</v>
       </c>
       <c r="F12" t="str">
-        <v>1204… → wk4 2012</v>
+        <v>0192… → Jan 1992</v>
       </c>
       <c r="G12" t="str">
-        <v>high</v>
+        <v>low</v>
       </c>
       <c r="H12" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="I12" t="str">
-        <v>serial matches none of the residential/light-commercial era templates (e.g. commercial applied units)</v>
+        <v/>
       </c>
       <c r="J12" t="str">
-        <v>https://www.building-center.org/trane-hvac-age/ | https://www.partstown.com/cm/resource-center/guides/gd2/trane-serial-number-lookup</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -2311,16 +2311,16 @@
         <v>HVAC</v>
       </c>
       <c r="C13" t="str">
-        <v>2002–2009</v>
+        <v>2010–present</v>
       </c>
       <c r="D13" t="str">
-        <v>N WW… (single-digit year)</v>
+        <v>YYWW…</v>
       </c>
       <c r="E13" t="str">
-        <v>digit 1 = last digit of year (era-bounded 2002-2009), 2-3 = week</v>
+        <v>digits 1-2 = year, 3-4 = week</v>
       </c>
       <c r="F13" t="str">
-        <v>752… → wk52 2007</v>
+        <v>1204… → wk4 2012</v>
       </c>
       <c r="G13" t="str">
         <v>high</v>
@@ -2329,10 +2329,10 @@
         <v>Yes</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>serial matches none of the residential/light-commercial era templates (e.g. commercial applied units)</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>https://www.building-center.org/trane-hvac-age/ | https://www.partstown.com/cm/resource-center/guides/gd2/trane-serial-number-lookup</v>
       </c>
     </row>
     <row r="14">
@@ -2343,16 +2343,16 @@
         <v>HVAC</v>
       </c>
       <c r="C14" t="str">
-        <v>1983–2001</v>
+        <v>2002–2009</v>
       </c>
       <c r="D14" t="str">
-        <v>[YearLetter]WW…</v>
+        <v>N WW… (single-digit year)</v>
       </c>
       <c r="E14" t="str">
-        <v>letter = year (W=1983…S=2001), next 2 digits = week</v>
+        <v>digit 1 = last digit of year (era-bounded 2002-2009), 2-3 = week</v>
       </c>
       <c r="F14" t="str">
-        <v>K23… → wk23 1995</v>
+        <v>752… → wk52 2007</v>
       </c>
       <c r="G14" t="str">
         <v>high</v>
@@ -2375,19 +2375,19 @@
         <v>HVAC</v>
       </c>
       <c r="C15" t="str">
-        <v>pre-1983 / commercial applied</v>
+        <v>1983–2001</v>
       </c>
       <c r="D15" t="str">
-        <v>varies</v>
+        <v>[YearLetter]WW…</v>
       </c>
       <c r="E15" t="str">
-        <v>no reliable template</v>
+        <v>letter = year (W=1983…S=2001), next 2 digits = week</v>
       </c>
       <c r="F15" t="str">
-        <v>0A250312-1-1 (DOAS) → abstain</v>
+        <v>K23… → wk23 1995</v>
       </c>
       <c r="G15" t="str">
-        <v>low</v>
+        <v>high</v>
       </c>
       <c r="H15" t="str">
         <v>Yes</v>
@@ -2401,54 +2401,54 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Daikin</v>
+        <v>Trane</v>
       </c>
       <c r="B16" t="str">
         <v>HVAC</v>
       </c>
       <c r="C16" t="str">
-        <v>Daikin-badged residential</v>
+        <v>pre-1983 / commercial applied</v>
       </c>
       <c r="D16" t="str">
-        <v>xxxxYYMM…</v>
+        <v>varies</v>
       </c>
       <c r="E16" t="str">
-        <v>ignore first 4 chars; chars 5-6 = year, 7-8 = month</v>
+        <v>no reliable template</v>
       </c>
       <c r="F16" t="str">
-        <v>….1209… → Sep 2012</v>
+        <v>0A250312-1-1 (DOAS) → abstain</v>
       </c>
       <c r="G16" t="str">
-        <v>medium</v>
+        <v>low</v>
       </c>
       <c r="H16" t="str">
         <v>Yes</v>
       </c>
       <c r="I16" t="str">
-        <v>McQuay applied lines (position varies) or non-matching shape → lookup</v>
+        <v/>
       </c>
       <c r="J16" t="str">
-        <v>https://inspectorhandbook.com/hvac/daikin | https://www.building-center.org/daikin-hvac-age/</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Lennox</v>
+        <v>Daikin</v>
       </c>
       <c r="B17" t="str">
         <v>HVAC</v>
       </c>
       <c r="C17" t="str">
-        <v>classic 1974–present</v>
+        <v>Daikin-badged residential</v>
       </c>
       <c r="D17" t="str">
-        <v>PPYY[MonthLetter]nnnnn</v>
+        <v>xxxxYYMM…</v>
       </c>
       <c r="E17" t="str">
-        <v>digits 1-2 = plant, 3-4 = year, 5th char = month letter (A=Jan…M=Dec, no I)</v>
+        <v>ignore first 4 chars; chars 5-6 = year, 7-8 = month</v>
       </c>
       <c r="F17" t="str">
-        <v>5621M99989 → Dec 2021</v>
+        <v>….1209… → Sep 2012</v>
       </c>
       <c r="G17" t="str">
         <v>medium</v>
@@ -2457,42 +2457,42 @@
         <v>Yes</v>
       </c>
       <c r="I17" t="str">
-        <v>serial not in classic PPYY[letter] shape</v>
+        <v>McQuay applied lines (position varies) or non-matching shape → lookup</v>
       </c>
       <c r="J17" t="str">
-        <v>https://www.building-center.org/lennox-hvac-age/ | https://www.pickhvac.com/hvac/age-serial-number/lennox/</v>
+        <v>https://inspectorhandbook.com/hvac/daikin | https://www.building-center.org/daikin-hvac-age/</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Manitowoc Ice</v>
+        <v>Lennox</v>
       </c>
       <c r="B18" t="str">
-        <v>Ice machines</v>
+        <v>HVAC</v>
       </c>
       <c r="C18" t="str">
-        <v>pre-2006</v>
+        <v>classic 1974–present</v>
       </c>
       <c r="D18" t="str">
-        <v>YYMMnnnnn</v>
+        <v>PPYY[MonthLetter]nnnnn</v>
       </c>
       <c r="E18" t="str">
-        <v>digits 1-2 = year, 3-4 = month</v>
+        <v>digits 1-2 = plant, 3-4 = year, 5th char = month letter (A=Jan…M=Dec, no I)</v>
       </c>
       <c r="F18" t="str">
-        <v>050164303 → Jan 2005</v>
+        <v>5621M99989 → Dec 2021</v>
       </c>
       <c r="G18" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="H18" t="str">
         <v>Yes</v>
       </c>
       <c r="I18" t="str">
-        <v>first-4-digit block gives month &gt;12, or a post-2006 sequential serial with no MFG DT captured</v>
+        <v>serial not in classic PPYY[letter] shape</v>
       </c>
       <c r="J18" t="str">
-        <v>https://www.easyice.com/how-to-read-a-manitowoc-serial-number | https://www.icemachineclearance.com/blog/manitowoc-ice-machine-serial-numbers/</v>
+        <v>https://www.building-center.org/lennox-hvac-age/ | https://www.pickhvac.com/hvac/age-serial-number/lennox/</v>
       </c>
     </row>
     <row r="19">
@@ -2503,16 +2503,16 @@
         <v>Ice machines</v>
       </c>
       <c r="C19" t="str">
-        <v>2006+</v>
+        <v>pre-2006</v>
       </c>
       <c r="D19" t="str">
-        <v>sequential serial + separate "MFG DT" YYMM plate stamp</v>
+        <v>YYMMnnnnn</v>
       </c>
       <c r="E19" t="str">
-        <v>serial not date-bearing; read the MFG DT field</v>
+        <v>digits 1-2 = year, 3-4 = month</v>
       </c>
       <c r="F19" t="str">
-        <v>MFG DT 0608 → Aug 2006</v>
+        <v>050164303 → Jan 2005</v>
       </c>
       <c r="G19" t="str">
         <v>high</v>
@@ -2521,30 +2521,30 @@
         <v>Yes</v>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>first-4-digit block gives month &gt;12, or a post-2006 sequential serial with no MFG DT captured</v>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>https://www.easyice.com/how-to-read-a-manitowoc-serial-number | https://www.icemachineclearance.com/blog/manitowoc-ice-machine-serial-numbers/</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Scotsman</v>
+        <v>Manitowoc Ice</v>
       </c>
       <c r="B20" t="str">
         <v>Ice machines</v>
       </c>
       <c r="C20" t="str">
-        <v>after May 2004</v>
+        <v>2006+</v>
       </c>
       <c r="D20" t="str">
-        <v>YYMMxxxx…</v>
+        <v>sequential serial + separate "MFG DT" YYMM plate stamp</v>
       </c>
       <c r="E20" t="str">
-        <v>digits 1-2 = year, 3-4 = month; digits 5-8 = site ID</v>
+        <v>serial not date-bearing; read the MFG DT field</v>
       </c>
       <c r="F20" t="str">
-        <v>0711… → Nov 2007</v>
+        <v>MFG DT 0608 → Aug 2006</v>
       </c>
       <c r="G20" t="str">
         <v>high</v>
@@ -2553,10 +2553,10 @@
         <v>Yes</v>
       </c>
       <c r="I20" t="str">
-        <v>pre-2004 year letter cannot be pinned to a decade; trailing block matches neither pattern</v>
+        <v/>
       </c>
       <c r="J20" t="str">
-        <v>https://www.partstown.com/cm/resource-center/guides/gd2/how-to-read-a-scotsman-serial-number</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -2567,112 +2567,112 @@
         <v>Ice machines</v>
       </c>
       <c r="C21" t="str">
-        <v>through May 2004</v>
+        <v>after May 2004</v>
       </c>
       <c r="D21" t="str">
-        <v>…MM[YearLetter]</v>
+        <v>YYMMxxxx…</v>
       </c>
       <c r="E21" t="str">
-        <v>last 3 chars: 2-digit OFFSET month (07=Jan…12=Jun,01=Jul…06=Dec) + cycling year letter</v>
+        <v>digits 1-2 = year, 3-4 = month; digits 5-8 = site ID</v>
       </c>
       <c r="F21" t="str">
-        <v>…09D → Mar 2002</v>
+        <v>0711… → Nov 2007</v>
       </c>
       <c r="G21" t="str">
-        <v>medium</v>
+        <v>high</v>
       </c>
       <c r="H21" t="str">
         <v>Yes</v>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>pre-2004 year letter cannot be pinned to a decade; trailing block matches neither pattern</v>
       </c>
       <c r="J21" t="str">
-        <v/>
+        <v>https://www.partstown.com/cm/resource-center/guides/gd2/how-to-read-a-scotsman-serial-number</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Grundfos</v>
+        <v>Scotsman</v>
       </c>
       <c r="B22" t="str">
-        <v>Pumps</v>
+        <v>Ice machines</v>
       </c>
       <c r="C22" t="str">
-        <v>modern nameplate</v>
+        <v>through May 2004</v>
       </c>
       <c r="D22" t="str">
-        <v>PC = YYWW (production code, often circled)</v>
+        <v>…MM[YearLetter]</v>
       </c>
       <c r="E22" t="str">
-        <v>digits 1-2 = year, 3-4 = ISO week</v>
+        <v>last 3 chars: 2-digit OFFSET month (07=Jan…12=Jun,01=Jul…06=Dec) + cycling year letter</v>
       </c>
       <c r="F22" t="str">
-        <v>PC 0833 → wk33 2008</v>
+        <v>…09D → Mar 2002</v>
       </c>
       <c r="G22" t="str">
-        <v>high</v>
+        <v>medium</v>
       </c>
       <c r="H22" t="str">
         <v>Yes</v>
       </c>
       <c r="I22" t="str">
-        <v>century unclear (2-digit year), or no PC code present</v>
+        <v/>
       </c>
       <c r="J22" t="str">
-        <v>https://www.grundfos.com/us/support/how-to-guides/finding-a-product-number-on-a-pump-nameplate</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Armstrong Fluid Technology</v>
+        <v>Grundfos</v>
       </c>
       <c r="B23" t="str">
         <v>Pumps</v>
       </c>
       <c r="C23" t="str">
-        <v>circulators</v>
+        <v>modern nameplate</v>
       </c>
       <c r="D23" t="str">
-        <v>YYMM (4-digit date/serial code)</v>
+        <v>PC = YYWW (production code, often circled)</v>
       </c>
       <c r="E23" t="str">
-        <v>digits 1-2 = year, 3-4 = month</v>
+        <v>digits 1-2 = year, 3-4 = ISO week</v>
       </c>
       <c r="F23" t="str">
-        <v>0106 → Jun 2001</v>
+        <v>PC 0833 → wk33 2008</v>
       </c>
       <c r="G23" t="str">
-        <v>medium</v>
+        <v>high</v>
       </c>
       <c r="H23" t="str">
         <v>Yes</v>
       </c>
       <c r="I23" t="str">
-        <v>large engineered/special-material pumps use a plain serial (no date) → lookup</v>
+        <v>century unclear (2-digit year), or no PC code present</v>
       </c>
       <c r="J23" t="str">
-        <v>https://www.nationalpumpsupply.com/content/pdf/armstrong-pump-circulator-pump-parts-list.pdf</v>
+        <v>https://www.grundfos.com/us/support/how-to-guides/finding-a-product-number-on-a-pump-nameplate</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Wilo</v>
+        <v>Armstrong Fluid Technology</v>
       </c>
       <c r="B24" t="str">
         <v>Pumps</v>
       </c>
       <c r="C24" t="str">
-        <v>nameplate date code</v>
+        <v>circulators</v>
       </c>
       <c r="D24" t="str">
-        <v>YYWW</v>
+        <v>YYMM (4-digit date/serial code)</v>
       </c>
       <c r="E24" t="str">
-        <v>digits 1-2 = year, 3-4 = week</v>
+        <v>digits 1-2 = year, 3-4 = month</v>
       </c>
       <c r="F24" t="str">
-        <v>2423 → wk23 2024</v>
+        <v>0106 → Jun 2001</v>
       </c>
       <c r="G24" t="str">
         <v>medium</v>
@@ -2681,30 +2681,30 @@
         <v>Yes</v>
       </c>
       <c r="I24" t="str">
-        <v>date field layout not obvious on longer serials</v>
+        <v>large engineered/special-material pumps use a plain serial (no date) → lookup</v>
       </c>
       <c r="J24" t="str">
-        <v>https://cms.media.wilo.com/cdndoc/wilo666890/8475454/wilo666890.pdf</v>
+        <v>https://www.nationalpumpsupply.com/content/pdf/armstrong-pump-circulator-pump-parts-list.pdf</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Baldor (ABB)</v>
+        <v>Wilo</v>
       </c>
       <c r="B25" t="str">
-        <v>Electric motors</v>
+        <v>Pumps</v>
       </c>
       <c r="C25" t="str">
-        <v>modern NEMA serial</v>
+        <v>nameplate date code</v>
       </c>
       <c r="D25" t="str">
-        <v>[Plant]YYMMDD…</v>
+        <v>YYWW</v>
       </c>
       <c r="E25" t="str">
-        <v>skip plant letter; next 2 = year, 2 = month, 2 = day</v>
+        <v>digits 1-2 = year, 3-4 = week</v>
       </c>
       <c r="F25" t="str">
-        <v>C1701181132 → 2017-01-18</v>
+        <v>2423 → wk23 2024</v>
       </c>
       <c r="G25" t="str">
         <v>medium</v>
@@ -2713,10 +2713,10 @@
         <v>Yes</v>
       </c>
       <c r="I25" t="str">
-        <v>serial not in plant+YYMMDD shape, or only a legacy grid code present</v>
+        <v>date field layout not obvious on longer serials</v>
       </c>
       <c r="J25" t="str">
-        <v>https://www.pooleyinc.com/wp-content/uploads/Baldor-Dodge-Mfr-Date-Code-Chart.pdf</v>
+        <v>https://cms.media.wilo.com/cdndoc/wilo666890/8475454/wilo666890.pdf</v>
       </c>
     </row>
     <row r="26">
@@ -2727,33 +2727,65 @@
         <v>Electric motors</v>
       </c>
       <c r="C26" t="str">
+        <v>modern NEMA serial</v>
+      </c>
+      <c r="D26" t="str">
+        <v>[Plant]YYMMDD…</v>
+      </c>
+      <c r="E26" t="str">
+        <v>skip plant letter; next 2 = year, 2 = month, 2 = day</v>
+      </c>
+      <c r="F26" t="str">
+        <v>C1701181132 → 2017-01-18</v>
+      </c>
+      <c r="G26" t="str">
+        <v>medium</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="I26" t="str">
+        <v>serial not in plant+YYMMDD shape, or only a legacy grid code present</v>
+      </c>
+      <c r="J26" t="str">
+        <v>https://www.pooleyinc.com/wp-content/uploads/Baldor-Dodge-Mfr-Date-Code-Chart.pdf</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Baldor (ABB)</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Electric motors</v>
+      </c>
+      <c r="C27" t="str">
         <v>legacy Dodge grid code</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D27" t="str">
         <v>2-char grid code</v>
       </c>
-      <c r="E26" t="str">
+      <c r="E27" t="str">
         <v>reverse-map via Baldor-Dodge date-code chart (not computable)</v>
       </c>
-      <c r="F26" t="str">
+      <c r="F27" t="str">
         <v>—</v>
       </c>
-      <c r="G26" t="str">
+      <c r="G27" t="str">
         <v>low</v>
       </c>
-      <c r="H26" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="I26" t="str">
+      <c r="H27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="I27" t="str">
         <v/>
       </c>
-      <c r="J26" t="str">
+      <c r="J27" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J27"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Validate Alliance/IPSO date code against manufacturer; promote to high
Alliance warranty portal confirmed all three Boca Raton washer-extractors:
  40F002829FH  → ship 5/26/2016   (decoded Apr 2016)  ✓ 2016
  280FX001342FY → ship 12/21/2016 (decoded Nov 2016)  ✓ 2016
  40F003349MK  → ship 7/1/2019    (decoded May 2019)  ✓ 2019
The letter code decodes the MANUFACTURE date; Alliance ships ~1-2 months
later, so decoded month runs just ahead of ship date in every case.

- serialDecoder.js / brands.js: IPSO trailing-letter rule promoted
  medium → high (manufacturer-validated).
- groundTruth.js: added the 3 validated serials.
- Pilot now 12/12 = 100% precision across 18 real rows.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Kn8R8jTNya2ZZLsLje6xJ
</commit_message>
<xml_diff>
--- a/docs/Serial-Decoding-Reference.xlsx
+++ b/docs/Serial-Decoding-Reference.xlsx
@@ -1997,13 +1997,13 @@
         <v>…[YearLetter][MonthLetter]</v>
       </c>
       <c r="E3" t="str">
-        <v>date is the LAST two letters: penultimate = year (cycles ~20 yrs: …D=2015,F=2016,H=2017,K=2018,M=2019,Q=2020), last = month (two letters/month: Apr=G/H, May=J/K, Nov=V/Y). Leading digits are a plant/sequence code, NOT the date</v>
+        <v>date is the LAST two letters: penultimate = year (cycles ~20 yrs: …D=2015,F=2016,H=2017,K=2018,M=2019,Q=2020), last = month (two letters/month: Apr=G/H, May=J/K, Nov=V/Y). Leading digits are a plant/sequence code, NOT the date. VALIDATED vs Alliance ship dates (decodes manufacture date; ship ~1-2 mo later)</v>
       </c>
       <c r="F3" t="str">
-        <v>40F002829FH → Apr 2016; 40F003349MK → May 2019</v>
+        <v>40F002829FH → Apr 2016 (Alliance ship 5/26/2016); 40F003349MK → May 2019 (ship 7/1/2019)</v>
       </c>
       <c r="G3" t="str">
-        <v>medium</v>
+        <v>high</v>
       </c>
       <c r="H3" t="str">
         <v>Yes</v>

</xml_diff>